<commit_message>
feature: csv for testing that allow to run workflow (except level2)
</commit_message>
<xml_diff>
--- a/R/tunaatlas_scripts/pre-harmonization/iccat/effort/data/t2ce_ETRO-PS1991-2024_bySchool_v1.xlsx
+++ b/R/tunaatlas_scripts/pre-harmonization/iccat/effort/data/t2ce_ETRO-PS1991-2024_bySchool_v1.xlsx
@@ -353,7 +353,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -380,85 +380,85 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Metadata</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Metadata</t>
+          <t>Time series start</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>1991</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Time series start</t>
+          <t>Time series end</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1991</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Time series end</t>
+          <t>Total years</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>34</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Total years</t>
+          <t>Number of records</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>329354</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Number of records</t>
+          <t>Number of fleets</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>329354</t>
+          <t>26</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Number of fleets</t>
+          <t>Number of flags</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Number of flags</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
         <is>
           <t>18</t>
         </is>
@@ -471,7 +471,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AG11"/>
+  <dimension ref="A1:AG21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -643,19 +643,19 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>2797</v>
+        <v>3666</v>
       </c>
       <c r="B2">
-        <v>509067</v>
+        <v>1280134</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>EU-España</t>
+          <t>St Vincent and Grenadines</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>EU.ESP-ES-ETRO</t>
+          <t>VCT-VC-ETRO</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -664,13 +664,13 @@
         </is>
       </c>
       <c r="F2">
-        <v>1994</v>
+        <v>1991</v>
       </c>
       <c r="G2">
         <v>1990</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -678,27 +678,27 @@
         </is>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="M2">
-        <v>1.5</v>
+        <v>-11.5</v>
       </c>
       <c r="N2">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>FAD</t>
+          <t>FSC</t>
         </is>
       </c>
       <c r="P2">
-        <v>13</v>
+        <v>12.2</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="R2">
-        <v>25.9</v>
+        <v>24</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -714,7 +714,7 @@
         </is>
       </c>
       <c r="T2">
-        <v>13</v>
+        <v>12.2</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
@@ -764,19 +764,19 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>2797</v>
+        <v>3762</v>
       </c>
       <c r="B3">
-        <v>509068</v>
+        <v>551876</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>EU-España</t>
+          <t>Curaçao</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>EU.ESP-ES-ETRO</t>
+          <t>CUW-CW-ETRO</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -785,13 +785,13 @@
         </is>
       </c>
       <c r="F3">
-        <v>1994</v>
+        <v>2001</v>
       </c>
       <c r="G3">
-        <v>1990</v>
+        <v>2000</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -799,19 +799,19 @@
         </is>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K3">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="L3">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="M3">
-        <v>0.5</v>
+        <v>-19.5</v>
       </c>
       <c r="N3">
-        <v>1.5</v>
+        <v>8.5</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="P3">
-        <v>13</v>
+        <v>25.1</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="R3">
-        <v>25.9</v>
+        <v>48</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="T3">
-        <v>13</v>
+        <v>25.1</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
@@ -843,7 +843,7 @@
         </is>
       </c>
       <c r="V3">
-        <v>0</v>
+        <v>2.48</v>
       </c>
       <c r="W3" t="inlineStr">
         <is>
@@ -859,13 +859,13 @@
         </is>
       </c>
       <c r="Z3">
-        <v>0</v>
+        <v>4240</v>
       </c>
       <c r="AA3">
         <v>0</v>
       </c>
       <c r="AB3">
-        <v>0</v>
+        <v>7380</v>
       </c>
       <c r="AC3">
         <v>0</v>
@@ -874,30 +874,30 @@
         <v>0</v>
       </c>
       <c r="AE3">
-        <v>0</v>
+        <v>31840</v>
       </c>
       <c r="AF3">
         <v>0</v>
       </c>
       <c r="AG3">
-        <v>0</v>
+        <v>43460</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>2797</v>
+        <v>5360</v>
       </c>
       <c r="B4">
-        <v>509069</v>
+        <v>1317242</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>EU-España</t>
+          <t>Curaçao</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>EU.ESP-ES-ETRO</t>
+          <t>CUW-CW-ETRO</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -906,13 +906,13 @@
         </is>
       </c>
       <c r="F4">
-        <v>1994</v>
+        <v>2012</v>
       </c>
       <c r="G4">
-        <v>1990</v>
+        <v>2010</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -920,27 +920,27 @@
         </is>
       </c>
       <c r="J4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L4">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="M4">
-        <v>2.5</v>
+        <v>7.5</v>
       </c>
       <c r="N4">
-        <v>1.5</v>
+        <v>-3.5</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>FAD</t>
+          <t>FSC</t>
         </is>
       </c>
       <c r="P4">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -948,7 +948,7 @@
         </is>
       </c>
       <c r="R4">
-        <v>25.9</v>
+        <v>48</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -956,7 +956,7 @@
         </is>
       </c>
       <c r="T4">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="V4">
-        <v>0</v>
+        <v>4.36</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
@@ -1006,19 +1006,19 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>2797</v>
+        <v>6141</v>
       </c>
       <c r="B5">
-        <v>509070</v>
+        <v>845164</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>EU-España</t>
+          <t>Côte d'Ivoire</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>EU.ESP-ES-ETRO</t>
+          <t>CIV-CI-ETRO</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1027,13 +1027,13 @@
         </is>
       </c>
       <c r="F5">
-        <v>1994</v>
+        <v>2014</v>
       </c>
       <c r="G5">
-        <v>1990</v>
+        <v>2010</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -1041,19 +1041,19 @@
         </is>
       </c>
       <c r="J5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L5">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="M5">
-        <v>0.5</v>
+        <v>-8.5</v>
       </c>
       <c r="N5">
-        <v>-0.5</v>
+        <v>-4.5</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1061,7 +1061,7 @@
         </is>
       </c>
       <c r="P5">
-        <v>13.1</v>
+        <v>12.2</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -1069,7 +1069,7 @@
         </is>
       </c>
       <c r="R5">
-        <v>25.9</v>
+        <v>24</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="T5">
-        <v>13.1</v>
+        <v>12.2</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
@@ -1101,13 +1101,13 @@
         </is>
       </c>
       <c r="Z5">
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="AA5">
         <v>0</v>
       </c>
       <c r="AB5">
-        <v>0</v>
+        <v>580</v>
       </c>
       <c r="AC5">
         <v>0</v>
@@ -1116,30 +1116,30 @@
         <v>0</v>
       </c>
       <c r="AE5">
-        <v>0</v>
+        <v>2210</v>
       </c>
       <c r="AF5">
         <v>0</v>
       </c>
       <c r="AG5">
-        <v>0</v>
+        <v>3010</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <v>2797</v>
+        <v>6142</v>
       </c>
       <c r="B6">
-        <v>509071</v>
+        <v>845701</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>EU-España</t>
+          <t>Guinée Rep</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>EU.ESP-ES-ETRO</t>
+          <t>GIN-GN-ETRO</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1148,13 +1148,13 @@
         </is>
       </c>
       <c r="F6">
-        <v>1994</v>
+        <v>2014</v>
       </c>
       <c r="G6">
-        <v>1990</v>
+        <v>2010</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -1162,19 +1162,19 @@
         </is>
       </c>
       <c r="J6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K6">
         <v>0</v>
       </c>
       <c r="L6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M6">
-        <v>1.5</v>
+        <v>-3.5</v>
       </c>
       <c r="N6">
-        <v>-0.5</v>
+        <v>0.5</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="P6">
-        <v>26.1</v>
+        <v>0</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="R6">
-        <v>51.8</v>
+        <v>24</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
         </is>
       </c>
       <c r="T6">
-        <v>26.1</v>
+        <v>0</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="X6">
-        <v>2.21</v>
+        <v>0</v>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
@@ -1248,19 +1248,19 @@
     </row>
     <row r="7">
       <c r="A7">
-        <v>2797</v>
+        <v>7158</v>
       </c>
       <c r="B7">
-        <v>509072</v>
+        <v>1043469</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>EU-España</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>EU.ESP-ES-ETRO</t>
+          <t>GHA-GH-ETRO-A</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1269,13 +1269,13 @@
         </is>
       </c>
       <c r="F7">
-        <v>1994</v>
+        <v>1996</v>
       </c>
       <c r="G7">
         <v>1990</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -1283,73 +1283,49 @@
         </is>
       </c>
       <c r="J7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K7">
         <v>0</v>
       </c>
       <c r="L7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="M7">
+        <v>-8.5</v>
+      </c>
+      <c r="N7">
+        <v>0.5</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>FAD</t>
+        </is>
+      </c>
+      <c r="P7">
+        <v>1.26</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>FISH.HOUR</t>
+        </is>
+      </c>
+      <c r="R7">
         <v>2.5</v>
       </c>
-      <c r="N7">
-        <v>-0.5</v>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>FAD</t>
-        </is>
-      </c>
-      <c r="P7">
-        <v>12.1</v>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>FISH.HOUR</t>
-        </is>
-      </c>
-      <c r="R7">
-        <v>24</v>
-      </c>
       <c r="S7" t="inlineStr">
         <is>
           <t>HOURS.SEA</t>
         </is>
       </c>
-      <c r="T7">
-        <v>12.1</v>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>Hours.STD</t>
-        </is>
-      </c>
-      <c r="V7">
-        <v>0</v>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>Hours.FAD</t>
-        </is>
-      </c>
-      <c r="X7">
-        <v>0</v>
-      </c>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>Hours.FSC</t>
-        </is>
-      </c>
       <c r="Z7">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="AA7">
         <v>0</v>
       </c>
       <c r="AB7">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="AC7">
         <v>0</v>
@@ -1358,30 +1334,30 @@
         <v>0</v>
       </c>
       <c r="AE7">
-        <v>0</v>
+        <v>151</v>
       </c>
       <c r="AF7">
         <v>0</v>
       </c>
       <c r="AG7">
-        <v>0</v>
+        <v>252</v>
       </c>
     </row>
     <row r="8">
       <c r="A8">
-        <v>2797</v>
+        <v>7214</v>
       </c>
       <c r="B8">
-        <v>509073</v>
+        <v>1148690</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>EU-España</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>EU.ESP-ES-ETRO</t>
+          <t>GTM-GT-ETRO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1390,13 +1366,13 @@
         </is>
       </c>
       <c r="F8">
-        <v>1994</v>
+        <v>2007</v>
       </c>
       <c r="G8">
-        <v>1990</v>
+        <v>2000</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -1404,35 +1380,35 @@
         </is>
       </c>
       <c r="J8">
+        <v>4</v>
+      </c>
+      <c r="K8">
+        <v>4</v>
+      </c>
+      <c r="L8">
+        <v>4</v>
+      </c>
+      <c r="M8">
+        <v>-4.5</v>
+      </c>
+      <c r="N8">
+        <v>4.5</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>FAD</t>
+        </is>
+      </c>
+      <c r="P8">
         <v>2</v>
       </c>
-      <c r="K8">
-        <v>1</v>
-      </c>
-      <c r="L8">
-        <v>0</v>
-      </c>
-      <c r="M8">
-        <v>0.5</v>
-      </c>
-      <c r="N8">
-        <v>-1.5</v>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>FAD</t>
-        </is>
-      </c>
-      <c r="P8">
-        <v>862.5</v>
-      </c>
       <c r="Q8" t="inlineStr">
         <is>
           <t>FISH.HOUR</t>
         </is>
       </c>
       <c r="R8">
-        <v>1732.9</v>
+        <v>14</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1440,7 +1416,7 @@
         </is>
       </c>
       <c r="T8">
-        <v>862.5</v>
+        <v>2.1</v>
       </c>
       <c r="U8" t="inlineStr">
         <is>
@@ -1448,7 +1424,7 @@
         </is>
       </c>
       <c r="V8">
-        <v>2.26</v>
+        <v>0</v>
       </c>
       <c r="W8" t="inlineStr">
         <is>
@@ -1456,7 +1432,7 @@
         </is>
       </c>
       <c r="X8">
-        <v>187.41</v>
+        <v>0</v>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
@@ -1464,13 +1440,13 @@
         </is>
       </c>
       <c r="Z8">
-        <v>1180</v>
+        <v>0</v>
       </c>
       <c r="AA8">
         <v>0</v>
       </c>
       <c r="AB8">
-        <v>4590</v>
+        <v>0</v>
       </c>
       <c r="AC8">
         <v>0</v>
@@ -1479,30 +1455,30 @@
         <v>0</v>
       </c>
       <c r="AE8">
-        <v>10440</v>
+        <v>0</v>
       </c>
       <c r="AF8">
         <v>0</v>
       </c>
       <c r="AG8">
-        <v>16210</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <v>2797</v>
+        <v>7214</v>
       </c>
       <c r="B9">
-        <v>509074</v>
+        <v>1338746</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>EU-España</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>EU.ESP-ES-ETRO</t>
+          <t>GTM-GT-ETRO</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1511,13 +1487,13 @@
         </is>
       </c>
       <c r="F9">
-        <v>1994</v>
+        <v>2007</v>
       </c>
       <c r="G9">
-        <v>1990</v>
+        <v>2000</v>
       </c>
       <c r="H9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -1531,21 +1507,21 @@
         <v>1</v>
       </c>
       <c r="L9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M9">
-        <v>1.5</v>
+        <v>5.5</v>
       </c>
       <c r="N9">
         <v>-1.5</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>FAD</t>
+          <t>FSC</t>
         </is>
       </c>
       <c r="P9">
-        <v>732.6</v>
+        <v>24</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1553,7 +1529,7 @@
         </is>
       </c>
       <c r="R9">
-        <v>1471.9</v>
+        <v>48</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1561,7 +1537,7 @@
         </is>
       </c>
       <c r="T9">
-        <v>732.6</v>
+        <v>24.4</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
@@ -1569,7 +1545,7 @@
         </is>
       </c>
       <c r="V9">
-        <v>4.33</v>
+        <v>0</v>
       </c>
       <c r="W9" t="inlineStr">
         <is>
@@ -1577,7 +1553,7 @@
         </is>
       </c>
       <c r="X9">
-        <v>120.11</v>
+        <v>0</v>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
@@ -1585,13 +1561,13 @@
         </is>
       </c>
       <c r="Z9">
-        <v>3340</v>
+        <v>0</v>
       </c>
       <c r="AA9">
         <v>0</v>
       </c>
       <c r="AB9">
-        <v>2520</v>
+        <v>0</v>
       </c>
       <c r="AC9">
         <v>0</v>
@@ -1600,30 +1576,30 @@
         <v>0</v>
       </c>
       <c r="AE9">
-        <v>2790</v>
+        <v>0</v>
       </c>
       <c r="AF9">
         <v>0</v>
       </c>
       <c r="AG9">
-        <v>8650</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <v>2797</v>
+        <v>7231</v>
       </c>
       <c r="B10">
-        <v>509075</v>
+        <v>1158333</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>EU-España</t>
+          <t>Curaçao</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>EU.ESP-ES-ETRO</t>
+          <t>CUW-CW-ETRO</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1632,13 +1608,13 @@
         </is>
       </c>
       <c r="F10">
-        <v>1994</v>
+        <v>2011</v>
       </c>
       <c r="G10">
-        <v>1990</v>
+        <v>2010</v>
       </c>
       <c r="H10">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1646,19 +1622,19 @@
         </is>
       </c>
       <c r="J10">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L10">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="M10">
-        <v>2.5</v>
+        <v>-8.5</v>
       </c>
       <c r="N10">
-        <v>-1.5</v>
+        <v>0.5</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1666,7 +1642,7 @@
         </is>
       </c>
       <c r="P10">
-        <v>78.7</v>
+        <v>12.1</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1674,7 +1650,7 @@
         </is>
       </c>
       <c r="R10">
-        <v>155.4</v>
+        <v>24</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1682,7 +1658,7 @@
         </is>
       </c>
       <c r="T10">
-        <v>78.7</v>
+        <v>12.1</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
@@ -1698,7 +1674,7 @@
         </is>
       </c>
       <c r="X10">
-        <v>2.17</v>
+        <v>0</v>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
@@ -1732,122 +1708,1140 @@
     </row>
     <row r="11">
       <c r="A11">
-        <v>2797</v>
+        <v>8138</v>
       </c>
       <c r="B11">
-        <v>509076</v>
+        <v>1572244</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>EU-France</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>EU.FRA-FR-ETRO</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="F11">
+        <v>2002</v>
+      </c>
+      <c r="G11">
+        <v>2000</v>
+      </c>
+      <c r="H11">
+        <v>6</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>1x1</t>
+        </is>
+      </c>
+      <c r="J11">
+        <v>1</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>3</v>
+      </c>
+      <c r="M11">
+        <v>3.5</v>
+      </c>
+      <c r="N11">
+        <v>0.5</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>FSC</t>
+        </is>
+      </c>
+      <c r="P11">
+        <v>39.086</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>FISH.HOUR</t>
+        </is>
+      </c>
+      <c r="R11">
+        <v>5</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>NO.SETS</t>
+        </is>
+      </c>
+      <c r="Z11">
+        <v>389814</v>
+      </c>
+      <c r="AA11">
+        <v>0</v>
+      </c>
+      <c r="AB11">
+        <v>19802</v>
+      </c>
+      <c r="AC11">
+        <v>0</v>
+      </c>
+      <c r="AD11">
+        <v>0</v>
+      </c>
+      <c r="AE11">
+        <v>0</v>
+      </c>
+      <c r="AF11">
+        <v>0</v>
+      </c>
+      <c r="AG11">
+        <v>409616</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>8140</v>
+      </c>
+      <c r="B12">
+        <v>1574603</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>EU-France</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>EU.FRA-FR-ETRO</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="F12">
+        <v>2004</v>
+      </c>
+      <c r="G12">
+        <v>2000</v>
+      </c>
+      <c r="H12">
+        <v>1</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>1x1</t>
+        </is>
+      </c>
+      <c r="J12">
+        <v>3</v>
+      </c>
+      <c r="K12">
+        <v>2</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12">
+        <v>-1.5</v>
+      </c>
+      <c r="N12">
+        <v>-2.5</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>FAD</t>
+        </is>
+      </c>
+      <c r="P12">
+        <v>12.2</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>FISH.HOUR</t>
+        </is>
+      </c>
+      <c r="R12">
+        <v>1</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>NO.SETS</t>
+        </is>
+      </c>
+      <c r="Z12">
+        <v>983</v>
+      </c>
+      <c r="AA12">
+        <v>0</v>
+      </c>
+      <c r="AB12">
+        <v>1074</v>
+      </c>
+      <c r="AC12">
+        <v>0</v>
+      </c>
+      <c r="AD12">
+        <v>0</v>
+      </c>
+      <c r="AE12">
+        <v>8086</v>
+      </c>
+      <c r="AF12">
+        <v>0</v>
+      </c>
+      <c r="AG12">
+        <v>10143</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>8209</v>
+      </c>
+      <c r="B13">
+        <v>1615552</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>GHA-GH-ETRO-P</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="F13">
+        <v>2013</v>
+      </c>
+      <c r="G13">
+        <v>2010</v>
+      </c>
+      <c r="H13">
+        <v>12</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>1x1</t>
+        </is>
+      </c>
+      <c r="J13">
+        <v>4</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="L13">
+        <v>9</v>
+      </c>
+      <c r="M13">
+        <v>-9.5</v>
+      </c>
+      <c r="N13">
+        <v>0.5</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>FAD</t>
+        </is>
+      </c>
+      <c r="P13">
+        <v>1</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>NO.SETS</t>
+        </is>
+      </c>
+      <c r="R13">
+        <v>1</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>SUC.SETS</t>
+        </is>
+      </c>
+      <c r="T13">
+        <v>1</v>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>D.FISH</t>
+        </is>
+      </c>
+      <c r="V13">
+        <v>24</v>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>HOURS.SEA</t>
+        </is>
+      </c>
+      <c r="X13">
+        <v>12</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>FISH.HOUR</t>
+        </is>
+      </c>
+      <c r="Z13">
+        <v>0</v>
+      </c>
+      <c r="AA13">
+        <v>0</v>
+      </c>
+      <c r="AB13">
+        <v>0</v>
+      </c>
+      <c r="AC13">
+        <v>0</v>
+      </c>
+      <c r="AD13">
+        <v>0</v>
+      </c>
+      <c r="AE13">
+        <v>10000</v>
+      </c>
+      <c r="AF13">
+        <v>0</v>
+      </c>
+      <c r="AG13">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>8226</v>
+      </c>
+      <c r="B14">
+        <v>1632361</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>GHA-GH-ETRO-A</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="F14">
+        <v>2019</v>
+      </c>
+      <c r="G14">
+        <v>2010</v>
+      </c>
+      <c r="H14">
+        <v>12</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>1x1</t>
+        </is>
+      </c>
+      <c r="J14">
+        <v>3</v>
+      </c>
+      <c r="K14">
+        <v>2</v>
+      </c>
+      <c r="L14">
+        <v>15</v>
+      </c>
+      <c r="M14">
+        <v>-15.5</v>
+      </c>
+      <c r="N14">
+        <v>-2.5</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>FAD</t>
+        </is>
+      </c>
+      <c r="P14">
+        <v>1</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>NO.SETS</t>
+        </is>
+      </c>
+      <c r="R14">
+        <v>1</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>SUC.SETS</t>
+        </is>
+      </c>
+      <c r="T14">
+        <v>1</v>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>D.FISH</t>
+        </is>
+      </c>
+      <c r="V14">
+        <v>24</v>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>HOURS.SEA</t>
+        </is>
+      </c>
+      <c r="X14">
+        <v>12</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>FISH.HOUR</t>
+        </is>
+      </c>
+      <c r="Z14">
+        <v>4000</v>
+      </c>
+      <c r="AA14">
+        <v>0</v>
+      </c>
+      <c r="AB14">
+        <v>0</v>
+      </c>
+      <c r="AC14">
+        <v>0</v>
+      </c>
+      <c r="AD14">
+        <v>0</v>
+      </c>
+      <c r="AE14">
+        <v>11000</v>
+      </c>
+      <c r="AF14">
+        <v>0</v>
+      </c>
+      <c r="AG14">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>8400</v>
+      </c>
+      <c r="B15">
+        <v>1684417</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
           <t>EU-España</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>EU.ESP-ES-ETRO</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="F11">
-        <v>1994</v>
-      </c>
-      <c r="G11">
+      <c r="F15">
+        <v>1993</v>
+      </c>
+      <c r="G15">
         <v>1990</v>
       </c>
-      <c r="H11">
+      <c r="H15">
+        <v>5</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>1x1</t>
+        </is>
+      </c>
+      <c r="J15">
+        <v>4</v>
+      </c>
+      <c r="K15">
+        <v>9</v>
+      </c>
+      <c r="L15">
+        <v>18</v>
+      </c>
+      <c r="M15">
+        <v>-18.5</v>
+      </c>
+      <c r="N15">
+        <v>9.5</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="P15">
+        <v>12.5</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>FISH.HOUR</t>
+        </is>
+      </c>
+      <c r="R15">
+        <v>24</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>HOURS.SEA</t>
+        </is>
+      </c>
+      <c r="T15">
+        <v>12.4</v>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Hours.STD</t>
+        </is>
+      </c>
+      <c r="V15">
+        <v>0</v>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Hours.FAD</t>
+        </is>
+      </c>
+      <c r="X15">
+        <v>0</v>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>Hours.FSC</t>
+        </is>
+      </c>
+      <c r="Z15">
+        <v>0</v>
+      </c>
+      <c r="AA15">
+        <v>0</v>
+      </c>
+      <c r="AB15">
+        <v>0</v>
+      </c>
+      <c r="AC15">
+        <v>0</v>
+      </c>
+      <c r="AD15">
+        <v>0</v>
+      </c>
+      <c r="AE15">
+        <v>0</v>
+      </c>
+      <c r="AF15">
+        <v>0</v>
+      </c>
+      <c r="AG15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>8921</v>
+      </c>
+      <c r="B16">
+        <v>1797402</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>El Salvador</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>SLV-SV-ETRO</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="F16">
+        <v>2017</v>
+      </c>
+      <c r="G16">
+        <v>2010</v>
+      </c>
+      <c r="H16">
+        <v>9</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>1x1</t>
+        </is>
+      </c>
+      <c r="J16">
+        <v>4</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>10</v>
+      </c>
+      <c r="M16">
+        <v>-10.5</v>
+      </c>
+      <c r="N16">
+        <v>0.5</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>FAD</t>
+        </is>
+      </c>
+      <c r="P16">
         <v>1</v>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>NO.SETS</t>
+        </is>
+      </c>
+      <c r="R16">
+        <v>1</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>SUC.SETS</t>
+        </is>
+      </c>
+      <c r="Z16">
+        <v>730</v>
+      </c>
+      <c r="AA16">
+        <v>0</v>
+      </c>
+      <c r="AB16">
+        <v>660</v>
+      </c>
+      <c r="AC16">
+        <v>0</v>
+      </c>
+      <c r="AD16">
+        <v>0</v>
+      </c>
+      <c r="AE16">
+        <v>5380</v>
+      </c>
+      <c r="AF16">
+        <v>0</v>
+      </c>
+      <c r="AG16">
+        <v>6770</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>8934</v>
+      </c>
+      <c r="B17">
+        <v>1805250</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>EU-España</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>EU.ESP-ES-ETRO</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="F17">
+        <v>2016</v>
+      </c>
+      <c r="G17">
+        <v>2010</v>
+      </c>
+      <c r="H17">
+        <v>6</v>
+      </c>
+      <c r="I17" t="inlineStr">
         <is>
           <t>1x1</t>
         </is>
       </c>
-      <c r="J11">
+      <c r="J17">
+        <v>2</v>
+      </c>
+      <c r="K17">
         <v>3</v>
       </c>
-      <c r="K11">
+      <c r="L17">
+        <v>10</v>
+      </c>
+      <c r="M17">
+        <v>10.5</v>
+      </c>
+      <c r="N17">
+        <v>-3.5</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>FSC</t>
+        </is>
+      </c>
+      <c r="P17">
+        <v>3</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>NO.SETS</t>
+        </is>
+      </c>
+      <c r="R17">
+        <v>11.9</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>FISH.HOUR</t>
+        </is>
+      </c>
+      <c r="Z17">
+        <v>23080</v>
+      </c>
+      <c r="AA17">
+        <v>0</v>
+      </c>
+      <c r="AB17">
+        <v>3680</v>
+      </c>
+      <c r="AC17">
+        <v>0</v>
+      </c>
+      <c r="AD17">
+        <v>0</v>
+      </c>
+      <c r="AE17">
+        <v>72390</v>
+      </c>
+      <c r="AF17">
+        <v>0</v>
+      </c>
+      <c r="AG17">
+        <v>99150</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>8968</v>
+      </c>
+      <c r="B18">
+        <v>1821993</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>CUW-CW-ETRO</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="F18">
+        <v>2019</v>
+      </c>
+      <c r="G18">
+        <v>2010</v>
+      </c>
+      <c r="H18">
+        <v>8</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>1x1</t>
+        </is>
+      </c>
+      <c r="J18">
+        <v>4</v>
+      </c>
+      <c r="K18">
+        <v>18</v>
+      </c>
+      <c r="L18">
+        <v>18</v>
+      </c>
+      <c r="M18">
+        <v>-18.5</v>
+      </c>
+      <c r="N18">
+        <v>18.5</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>FAD</t>
+        </is>
+      </c>
+      <c r="P18">
+        <v>4</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>NO.SETS</t>
+        </is>
+      </c>
+      <c r="R18">
+        <v>3</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>SUC.SETS</t>
+        </is>
+      </c>
+      <c r="Z18">
+        <v>30720</v>
+      </c>
+      <c r="AA18">
+        <v>0</v>
+      </c>
+      <c r="AB18">
+        <v>20150</v>
+      </c>
+      <c r="AC18">
+        <v>0</v>
+      </c>
+      <c r="AD18">
+        <v>0</v>
+      </c>
+      <c r="AE18">
+        <v>358260</v>
+      </c>
+      <c r="AF18">
+        <v>0</v>
+      </c>
+      <c r="AG18">
+        <v>409130</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>9523</v>
+      </c>
+      <c r="B19">
+        <v>1946627</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Guatemala</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>GTM-GT-ETRO</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="F19">
+        <v>2023</v>
+      </c>
+      <c r="G19">
+        <v>2020</v>
+      </c>
+      <c r="H19">
+        <v>12</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>1x1</t>
+        </is>
+      </c>
+      <c r="J19">
+        <v>2</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19">
         <v>1</v>
       </c>
-      <c r="L11">
-        <v>21</v>
-      </c>
-      <c r="M11">
-        <v>-21.5</v>
-      </c>
-      <c r="N11">
+      <c r="M19">
+        <v>1.5</v>
+      </c>
+      <c r="N19">
+        <v>-0.5</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>FSC</t>
+        </is>
+      </c>
+      <c r="P19">
+        <v>1</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>NO.SETS</t>
+        </is>
+      </c>
+      <c r="R19">
+        <v>1</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>SUC.SETS</t>
+        </is>
+      </c>
+      <c r="Z19">
+        <v>21650</v>
+      </c>
+      <c r="AA19">
+        <v>0</v>
+      </c>
+      <c r="AB19">
+        <v>1330</v>
+      </c>
+      <c r="AC19">
+        <v>0</v>
+      </c>
+      <c r="AD19">
+        <v>0</v>
+      </c>
+      <c r="AE19">
+        <v>0</v>
+      </c>
+      <c r="AF19">
+        <v>0</v>
+      </c>
+      <c r="AG19">
+        <v>22980</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>9984</v>
+      </c>
+      <c r="B20">
+        <v>2012805</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>GHA-GH-ETRO-A</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="F20">
+        <v>2022</v>
+      </c>
+      <c r="G20">
+        <v>2020</v>
+      </c>
+      <c r="H20">
+        <v>9</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>1x1</t>
+        </is>
+      </c>
+      <c r="J20">
+        <v>3</v>
+      </c>
+      <c r="K20">
+        <v>3</v>
+      </c>
+      <c r="L20">
+        <v>13</v>
+      </c>
+      <c r="M20">
+        <v>-13.5</v>
+      </c>
+      <c r="N20">
+        <v>-3.5</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>FAD</t>
+        </is>
+      </c>
+      <c r="P20">
+        <v>3</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>NO.SETS</t>
+        </is>
+      </c>
+      <c r="R20">
+        <v>1.16</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>D.FISH</t>
+        </is>
+      </c>
+      <c r="Z20">
+        <v>31000</v>
+      </c>
+      <c r="AA20">
+        <v>0</v>
+      </c>
+      <c r="AB20">
+        <v>0</v>
+      </c>
+      <c r="AC20">
+        <v>0</v>
+      </c>
+      <c r="AD20">
+        <v>0</v>
+      </c>
+      <c r="AE20">
+        <v>84000</v>
+      </c>
+      <c r="AF20">
+        <v>0</v>
+      </c>
+      <c r="AG20">
+        <v>115000</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>9987</v>
+      </c>
+      <c r="B21">
+        <v>2015317</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>GHA-GH-ETRO-A</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="F21">
+        <v>2023</v>
+      </c>
+      <c r="G21">
+        <v>2020</v>
+      </c>
+      <c r="H21">
+        <v>10</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>1x1</t>
+        </is>
+      </c>
+      <c r="J21">
+        <v>4</v>
+      </c>
+      <c r="K21">
+        <v>4</v>
+      </c>
+      <c r="L21">
+        <v>1</v>
+      </c>
+      <c r="M21">
         <v>-1.5</v>
       </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>FAD</t>
-        </is>
-      </c>
-      <c r="P11">
-        <v>13.1</v>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>FISH.HOUR</t>
-        </is>
-      </c>
-      <c r="R11">
-        <v>25.9</v>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>HOURS.SEA</t>
-        </is>
-      </c>
-      <c r="T11">
-        <v>13.1</v>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>Hours.STD</t>
-        </is>
-      </c>
-      <c r="V11">
-        <v>0</v>
-      </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>Hours.FAD</t>
-        </is>
-      </c>
-      <c r="X11">
-        <v>0</v>
-      </c>
-      <c r="Y11" t="inlineStr">
-        <is>
-          <t>Hours.FSC</t>
-        </is>
-      </c>
-      <c r="Z11">
-        <v>0</v>
-      </c>
-      <c r="AA11">
-        <v>0</v>
-      </c>
-      <c r="AB11">
-        <v>0</v>
-      </c>
-      <c r="AC11">
-        <v>0</v>
-      </c>
-      <c r="AD11">
-        <v>0</v>
-      </c>
-      <c r="AE11">
-        <v>0</v>
-      </c>
-      <c r="AF11">
-        <v>0</v>
-      </c>
-      <c r="AG11">
+      <c r="N21">
+        <v>4.5</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="P21">
+        <v>0</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>NO.SETS</t>
+        </is>
+      </c>
+      <c r="R21">
+        <v>3</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>D.FISH</t>
+        </is>
+      </c>
+      <c r="Z21">
+        <v>0</v>
+      </c>
+      <c r="AA21">
+        <v>0</v>
+      </c>
+      <c r="AB21">
+        <v>0</v>
+      </c>
+      <c r="AC21">
+        <v>0</v>
+      </c>
+      <c r="AD21">
+        <v>0</v>
+      </c>
+      <c r="AE21">
+        <v>0</v>
+      </c>
+      <c r="AF21">
+        <v>0</v>
+      </c>
+      <c r="AG21">
         <v>0</v>
       </c>
     </row>
@@ -1858,7 +2852,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1920,90 +2914,108 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Sum of TOTAL</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>YearC</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sum of TOTAL</t>
+          <t>GearCode</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Flag</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>FleetCode</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>FishMode</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Eff1Type</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Eff2Type</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>YearC</t>
-        </is>
+          <t>2011</t>
+        </is>
+      </c>
+      <c r="H4">
+        <v>2021</v>
+      </c>
+      <c r="I4">
+        <v>2023</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GearCode</t>
+          <t>PS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Flag</t>
+          <t>EU-España</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>FleetCode</t>
+          <t>EU.ESP-ES-ETRO</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>FishMode</t>
+          <t>FAD</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Eff1Type</t>
+          <t>FISH.HOUR</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Eff2Type</t>
+          <t>HOURS.SEA</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>7560</t>
         </is>
       </c>
       <c r="H5">
-        <v>2021</v>
+        <v>43180</v>
       </c>
       <c r="I5">
-        <v>2023</v>
+        <v>82040</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>EU-España</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>EU.ESP-ES-ETRO</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>FAD</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>FISH.HOUR</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>HOURS.SEA</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -2015,24 +3027,6 @@
         <v>43180</v>
       </c>
       <c r="I6">
-        <v>82040</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>7560</t>
-        </is>
-      </c>
-      <c r="H7">
-        <v>43180</v>
-      </c>
-      <c r="I7">
         <v>82040</v>
       </c>
     </row>

</xml_diff>